<commit_message>
Set default target margin to 30% (site and Excel)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GHAGAmwRkNyFBmFrnvVcew
</commit_message>
<xml_diff>
--- a/Catalyst_IQ_Labs_AMS_Margin_Calculator_Weekly_-_V2.xlsx
+++ b/Catalyst_IQ_Labs_AMS_Margin_Calculator_Weekly_-_V2.xlsx
@@ -495,8 +495,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -944,405 +948,405 @@
   <dimension ref="A1:H38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="E4" s="3" t="s">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="E4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="8" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="9" t="n">
         <v>105</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="10" t="n">
+      <c r="F6" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="G6" s="10" t="n">
+      <c r="G6" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="H6" s="11" t="n">
+      <c r="H6" s="12" t="n">
         <v>189</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="F7" s="11" t="n">
         <v>21</v>
       </c>
-      <c r="G7" s="10" t="n">
+      <c r="G7" s="11" t="n">
         <v>29</v>
       </c>
-      <c r="H7" s="11" t="n">
+      <c r="H7" s="12" t="n">
         <v>179</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="12" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="C8" s="6" t="s">
+      <c r="B8" s="13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="F8" s="10" t="n">
+      <c r="F8" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="G8" s="10" t="n">
+      <c r="G8" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="H8" s="11" t="n">
+      <c r="H8" s="12" t="n">
         <v>169</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="13" t="n">
+      <c r="B9" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="15" t="n">
+      <c r="B10" s="16" t="n">
         <v>52</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="16" t="n">
+      <c r="B11" s="17" t="n">
         <v>50</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="17" t="str">
+      <c r="B14" s="18" t="str">
         <f aca="false">IF(AND($B$5&gt;=$F$6,$B$5&lt;=$G$8),INDEX($E$6:$E$8,MATCH($B$5,$F$6:$F$8,1)),"Out of range")</f>
         <v>Small</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="19" t="n">
+      <c r="B15" s="20" t="n">
         <f aca="false">IF(AND($B$5&gt;=$F$6,$B$5&lt;=$G$8),INDEX($H$6:$H$8,MATCH($B$5,$F$6:$F$8,1)),0)</f>
         <v>189</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="17" t="str">
+      <c r="B16" s="18" t="str">
         <f aca="false">IF(AND($B$5&gt;=$F$6,$B$5&lt;=$G$8),"OK – hours fall inside a tier","Hours outside "&amp;$F$6&amp;"–"&amp;$G$8&amp;" – no rate applies")</f>
         <v>OK – hours fall inside a tier</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="20" t="n">
+      <c r="B19" s="21" t="n">
         <f aca="false">B15*B5*$B$10/12</f>
         <v>16380</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="7" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="18" t="s">
+      <c r="A20" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="B20" s="19" t="n">
+      <c r="B20" s="20" t="n">
         <f aca="false">IF(B11&gt;0,CEILING(B19,B11),B19)</f>
         <v>16400</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="7" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B21" s="21" t="n">
+      <c r="B21" s="22" t="n">
         <f aca="false">B5*B9*$B$10/12</f>
         <v>86.6666666666667</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B22" s="20" t="n">
+      <c r="B22" s="21" t="n">
         <f aca="false">B6*B21</f>
         <v>9100</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B23" s="20" t="n">
+      <c r="B23" s="21" t="n">
         <f aca="false">B7*B21</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B24" s="20" t="n">
+      <c r="B24" s="21" t="n">
         <f aca="false">B19-B22</f>
         <v>7280</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B25" s="22" t="n">
+      <c r="B25" s="23" t="n">
         <f aca="false">IFERROR(B24/B19,0)</f>
         <v>0.444444444444444</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="18" t="s">
+      <c r="A26" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="B26" s="19" t="n">
+      <c r="B26" s="20" t="n">
         <f aca="false">B24-B23</f>
         <v>7280</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="18" t="s">
+      <c r="A27" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="B27" s="23" t="n">
+      <c r="B27" s="24" t="n">
         <f aca="false">IFERROR(B26/B19,0)</f>
         <v>0.444444444444444</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B28" s="17" t="str">
+      <c r="B28" s="18" t="str">
         <f aca="false">IF(B19=0,"No revenue",IF(B27&gt;=B8,"Meets target","Below target"))</f>
         <v>Meets target</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
+      <c r="A30" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
     </row>
     <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B31" s="20" t="n">
+      <c r="B31" s="21" t="n">
         <f aca="false">B19*12</f>
         <v>196560</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
+      <c r="A32" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B32" s="20" t="n">
+      <c r="B32" s="21" t="n">
         <f aca="false">B26*12</f>
         <v>87360</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B35" s="20" t="n">
+      <c r="B35" s="21" t="n">
         <f aca="false">IFERROR((B6+B7)*B9/(1-B8),0)</f>
-        <v>161.538461538462</v>
-      </c>
-      <c r="C35" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="C35" s="7" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
+      <c r="A36" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="B36" s="20" t="n">
+      <c r="B36" s="21" t="n">
         <f aca="false">B15-B35</f>
-        <v>27.4615384615385</v>
-      </c>
-      <c r="C36" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C36" s="7" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="4" t="s">
+      <c r="A37" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B37" s="21" t="n">
+      <c r="B37" s="22" t="n">
         <f aca="false">IFERROR(B15*B5*(1-B8)/(B6+B7),0)</f>
-        <v>23.4</v>
-      </c>
-      <c r="C37" s="6" t="s">
+        <v>25.2</v>
+      </c>
+      <c r="C37" s="7" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="4" t="s">
+      <c r="A38" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B38" s="21" t="n">
+      <c r="B38" s="22" t="n">
         <f aca="false">B37-B5*B9</f>
-        <v>3.4</v>
-      </c>
-      <c r="C38" s="6" t="s">
+        <v>5.2</v>
+      </c>
+      <c r="C38" s="7" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1446,401 +1450,401 @@
   <dimension ref="A1:J12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="24" t="s">
+      <c r="A4" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="B4" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="C4" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="D4" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="E4" s="24" t="s">
+      <c r="E4" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="F4" s="24" t="s">
+      <c r="F4" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="G4" s="24" t="s">
+      <c r="G4" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="H4" s="24" t="s">
+      <c r="H4" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="I4" s="24" t="str">
+      <c r="I4" s="25" t="str">
         <f aca="false">"Floor rate @ "&amp;TEXT('Margin Calculator'!$B$8,"0%")&amp;" ($/hr)"</f>
-        <v>Floor rate @ 35% ($/hr)</v>
-      </c>
-      <c r="J4" s="24" t="s">
+        <v>Floor rate @ 30% ($/hr)</v>
+      </c>
+      <c r="J4" s="25" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="25" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="B5" s="26" t="str">
+      <c r="B5" s="27" t="str">
         <f aca="false">IF(AND(A5&gt;='Margin Calculator'!$F$6,A5&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(A5,'Margin Calculator'!$F$6:$F$8,1)),"Out of range")</f>
         <v>Small</v>
       </c>
-      <c r="C5" s="27" t="n">
+      <c r="C5" s="28" t="n">
         <f aca="false">IF(AND(A5&gt;='Margin Calculator'!$F$6,A5&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(A5,'Margin Calculator'!$F$6:$F$8,1)),0)</f>
         <v>189</v>
       </c>
-      <c r="D5" s="27" t="n">
+      <c r="D5" s="28" t="n">
         <f aca="false">A5*C5*'Margin Calculator'!$B$10/12</f>
         <v>4095</v>
       </c>
-      <c r="E5" s="27" t="n">
+      <c r="E5" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$6*A5*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
         <v>2275</v>
       </c>
-      <c r="F5" s="27" t="n">
+      <c r="F5" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$7*A5*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
         <v>0</v>
       </c>
-      <c r="G5" s="27" t="n">
+      <c r="G5" s="28" t="n">
         <f aca="false">D5-E5-F5</f>
         <v>1820</v>
       </c>
-      <c r="H5" s="28" t="n">
+      <c r="H5" s="29" t="n">
         <f aca="false">IFERROR(G5/D5,0)</f>
         <v>0.444444444444444</v>
       </c>
-      <c r="I5" s="27" t="n">
+      <c r="I5" s="28" t="n">
         <f aca="false">IFERROR(('Margin Calculator'!$B$6+'Margin Calculator'!$B$7)*'Margin Calculator'!$B$9/(1-'Margin Calculator'!$B$8),0)</f>
-        <v>161.538461538462</v>
-      </c>
-      <c r="J5" s="26" t="str">
+        <v>150</v>
+      </c>
+      <c r="J5" s="27" t="str">
         <f aca="false">IF(D5=0,"–",IF(H5&gt;='Margin Calculator'!$B$8,"Yes","No"))</f>
         <v>Yes</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="25" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="B6" s="26" t="str">
+      <c r="B6" s="27" t="str">
         <f aca="false">IF(AND(A6&gt;='Margin Calculator'!$F$6,A6&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(A6,'Margin Calculator'!$F$6:$F$8,1)),"Out of range")</f>
         <v>Small</v>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="C6" s="28" t="n">
         <f aca="false">IF(AND(A6&gt;='Margin Calculator'!$F$6,A6&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(A6,'Margin Calculator'!$F$6:$F$8,1)),0)</f>
         <v>189</v>
       </c>
-      <c r="D6" s="27" t="n">
+      <c r="D6" s="28" t="n">
         <f aca="false">A6*C6*'Margin Calculator'!$B$10/12</f>
         <v>8190</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$6*A6*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
         <v>4550</v>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$7*A6*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
         <v>0</v>
       </c>
-      <c r="G6" s="27" t="n">
+      <c r="G6" s="28" t="n">
         <f aca="false">D6-E6-F6</f>
         <v>3640</v>
       </c>
-      <c r="H6" s="28" t="n">
+      <c r="H6" s="29" t="n">
         <f aca="false">IFERROR(G6/D6,0)</f>
         <v>0.444444444444444</v>
       </c>
-      <c r="I6" s="27" t="n">
+      <c r="I6" s="28" t="n">
         <f aca="false">IFERROR(('Margin Calculator'!$B$6+'Margin Calculator'!$B$7)*'Margin Calculator'!$B$9/(1-'Margin Calculator'!$B$8),0)</f>
-        <v>161.538461538462</v>
-      </c>
-      <c r="J6" s="26" t="str">
+        <v>150</v>
+      </c>
+      <c r="J6" s="27" t="str">
         <f aca="false">IF(D6=0,"–",IF(H6&gt;='Margin Calculator'!$B$8,"Yes","No"))</f>
         <v>Yes</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="25" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="26" t="n">
         <v>15</v>
       </c>
-      <c r="B7" s="26" t="str">
+      <c r="B7" s="27" t="str">
         <f aca="false">IF(AND(A7&gt;='Margin Calculator'!$F$6,A7&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(A7,'Margin Calculator'!$F$6:$F$8,1)),"Out of range")</f>
         <v>Small</v>
       </c>
-      <c r="C7" s="27" t="n">
+      <c r="C7" s="28" t="n">
         <f aca="false">IF(AND(A7&gt;='Margin Calculator'!$F$6,A7&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(A7,'Margin Calculator'!$F$6:$F$8,1)),0)</f>
         <v>189</v>
       </c>
-      <c r="D7" s="27" t="n">
+      <c r="D7" s="28" t="n">
         <f aca="false">A7*C7*'Margin Calculator'!$B$10/12</f>
         <v>12285</v>
       </c>
-      <c r="E7" s="27" t="n">
+      <c r="E7" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$6*A7*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
         <v>6825</v>
       </c>
-      <c r="F7" s="27" t="n">
+      <c r="F7" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$7*A7*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
         <v>0</v>
       </c>
-      <c r="G7" s="27" t="n">
+      <c r="G7" s="28" t="n">
         <f aca="false">D7-E7-F7</f>
         <v>5460</v>
       </c>
-      <c r="H7" s="28" t="n">
+      <c r="H7" s="29" t="n">
         <f aca="false">IFERROR(G7/D7,0)</f>
         <v>0.444444444444444</v>
       </c>
-      <c r="I7" s="27" t="n">
+      <c r="I7" s="28" t="n">
         <f aca="false">IFERROR(('Margin Calculator'!$B$6+'Margin Calculator'!$B$7)*'Margin Calculator'!$B$9/(1-'Margin Calculator'!$B$8),0)</f>
-        <v>161.538461538462</v>
-      </c>
-      <c r="J7" s="26" t="str">
+        <v>150</v>
+      </c>
+      <c r="J7" s="27" t="str">
         <f aca="false">IF(D7=0,"–",IF(H7&gt;='Margin Calculator'!$B$8,"Yes","No"))</f>
         <v>Yes</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="25" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="B8" s="26" t="str">
+      <c r="B8" s="27" t="str">
         <f aca="false">IF(AND(A8&gt;='Margin Calculator'!$F$6,A8&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(A8,'Margin Calculator'!$F$6:$F$8,1)),"Out of range")</f>
         <v>Small</v>
       </c>
-      <c r="C8" s="27" t="n">
+      <c r="C8" s="28" t="n">
         <f aca="false">IF(AND(A8&gt;='Margin Calculator'!$F$6,A8&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(A8,'Margin Calculator'!$F$6:$F$8,1)),0)</f>
         <v>189</v>
       </c>
-      <c r="D8" s="27" t="n">
+      <c r="D8" s="28" t="n">
         <f aca="false">A8*C8*'Margin Calculator'!$B$10/12</f>
         <v>16380</v>
       </c>
-      <c r="E8" s="27" t="n">
+      <c r="E8" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$6*A8*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
         <v>9100</v>
       </c>
-      <c r="F8" s="27" t="n">
+      <c r="F8" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$7*A8*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
         <v>0</v>
       </c>
-      <c r="G8" s="27" t="n">
+      <c r="G8" s="28" t="n">
         <f aca="false">D8-E8-F8</f>
         <v>7280</v>
       </c>
-      <c r="H8" s="28" t="n">
+      <c r="H8" s="29" t="n">
         <f aca="false">IFERROR(G8/D8,0)</f>
         <v>0.444444444444444</v>
       </c>
-      <c r="I8" s="27" t="n">
+      <c r="I8" s="28" t="n">
         <f aca="false">IFERROR(('Margin Calculator'!$B$6+'Margin Calculator'!$B$7)*'Margin Calculator'!$B$9/(1-'Margin Calculator'!$B$8),0)</f>
-        <v>161.538461538462</v>
-      </c>
-      <c r="J8" s="26" t="str">
+        <v>150</v>
+      </c>
+      <c r="J8" s="27" t="str">
         <f aca="false">IF(D8=0,"–",IF(H8&gt;='Margin Calculator'!$B$8,"Yes","No"))</f>
         <v>Yes</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="25" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="26" t="n">
         <v>25</v>
       </c>
-      <c r="B9" s="26" t="str">
+      <c r="B9" s="27" t="str">
         <f aca="false">IF(AND(A9&gt;='Margin Calculator'!$F$6,A9&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(A9,'Margin Calculator'!$F$6:$F$8,1)),"Out of range")</f>
         <v>Mid</v>
       </c>
-      <c r="C9" s="27" t="n">
+      <c r="C9" s="28" t="n">
         <f aca="false">IF(AND(A9&gt;='Margin Calculator'!$F$6,A9&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(A9,'Margin Calculator'!$F$6:$F$8,1)),0)</f>
         <v>179</v>
       </c>
-      <c r="D9" s="27" t="n">
+      <c r="D9" s="28" t="n">
         <f aca="false">A9*C9*'Margin Calculator'!$B$10/12</f>
         <v>19391.6666666667</v>
       </c>
-      <c r="E9" s="27" t="n">
+      <c r="E9" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$6*A9*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
         <v>11375</v>
       </c>
-      <c r="F9" s="27" t="n">
+      <c r="F9" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$7*A9*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
         <v>0</v>
       </c>
-      <c r="G9" s="27" t="n">
+      <c r="G9" s="28" t="n">
         <f aca="false">D9-E9-F9</f>
         <v>8016.66666666667</v>
       </c>
-      <c r="H9" s="28" t="n">
+      <c r="H9" s="29" t="n">
         <f aca="false">IFERROR(G9/D9,0)</f>
         <v>0.41340782122905</v>
       </c>
-      <c r="I9" s="27" t="n">
+      <c r="I9" s="28" t="n">
         <f aca="false">IFERROR(('Margin Calculator'!$B$6+'Margin Calculator'!$B$7)*'Margin Calculator'!$B$9/(1-'Margin Calculator'!$B$8),0)</f>
-        <v>161.538461538462</v>
-      </c>
-      <c r="J9" s="26" t="str">
+        <v>150</v>
+      </c>
+      <c r="J9" s="27" t="str">
         <f aca="false">IF(D9=0,"–",IF(H9&gt;='Margin Calculator'!$B$8,"Yes","No"))</f>
         <v>Yes</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="25" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="26" t="n">
         <v>30</v>
       </c>
-      <c r="B10" s="26" t="str">
+      <c r="B10" s="27" t="str">
         <f aca="false">IF(AND(A10&gt;='Margin Calculator'!$F$6,A10&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(A10,'Margin Calculator'!$F$6:$F$8,1)),"Out of range")</f>
         <v>Large</v>
       </c>
-      <c r="C10" s="27" t="n">
+      <c r="C10" s="28" t="n">
         <f aca="false">IF(AND(A10&gt;='Margin Calculator'!$F$6,A10&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(A10,'Margin Calculator'!$F$6:$F$8,1)),0)</f>
         <v>169</v>
       </c>
-      <c r="D10" s="27" t="n">
+      <c r="D10" s="28" t="n">
         <f aca="false">A10*C10*'Margin Calculator'!$B$10/12</f>
         <v>21970</v>
       </c>
-      <c r="E10" s="27" t="n">
+      <c r="E10" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$6*A10*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
         <v>13650</v>
       </c>
-      <c r="F10" s="27" t="n">
+      <c r="F10" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$7*A10*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
         <v>0</v>
       </c>
-      <c r="G10" s="27" t="n">
+      <c r="G10" s="28" t="n">
         <f aca="false">D10-E10-F10</f>
         <v>8320</v>
       </c>
-      <c r="H10" s="28" t="n">
+      <c r="H10" s="29" t="n">
         <f aca="false">IFERROR(G10/D10,0)</f>
         <v>0.378698224852071</v>
       </c>
-      <c r="I10" s="27" t="n">
+      <c r="I10" s="28" t="n">
         <f aca="false">IFERROR(('Margin Calculator'!$B$6+'Margin Calculator'!$B$7)*'Margin Calculator'!$B$9/(1-'Margin Calculator'!$B$8),0)</f>
-        <v>161.538461538462</v>
-      </c>
-      <c r="J10" s="26" t="str">
+        <v>150</v>
+      </c>
+      <c r="J10" s="27" t="str">
         <f aca="false">IF(D10=0,"–",IF(H10&gt;='Margin Calculator'!$B$8,"Yes","No"))</f>
         <v>Yes</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="25" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="B11" s="26" t="str">
+      <c r="B11" s="27" t="str">
         <f aca="false">IF(AND(A11&gt;='Margin Calculator'!$F$6,A11&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(A11,'Margin Calculator'!$F$6:$F$8,1)),"Out of range")</f>
         <v>Large</v>
       </c>
-      <c r="C11" s="27" t="n">
+      <c r="C11" s="28" t="n">
         <f aca="false">IF(AND(A11&gt;='Margin Calculator'!$F$6,A11&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(A11,'Margin Calculator'!$F$6:$F$8,1)),0)</f>
         <v>169</v>
       </c>
-      <c r="D11" s="27" t="n">
+      <c r="D11" s="28" t="n">
         <f aca="false">A11*C11*'Margin Calculator'!$B$10/12</f>
         <v>25631.6666666667</v>
       </c>
-      <c r="E11" s="27" t="n">
+      <c r="E11" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$6*A11*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
         <v>15925</v>
       </c>
-      <c r="F11" s="27" t="n">
+      <c r="F11" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$7*A11*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
         <v>0</v>
       </c>
-      <c r="G11" s="27" t="n">
+      <c r="G11" s="28" t="n">
         <f aca="false">D11-E11-F11</f>
         <v>9706.66666666667</v>
       </c>
-      <c r="H11" s="28" t="n">
+      <c r="H11" s="29" t="n">
         <f aca="false">IFERROR(G11/D11,0)</f>
         <v>0.378698224852071</v>
       </c>
-      <c r="I11" s="27" t="n">
+      <c r="I11" s="28" t="n">
         <f aca="false">IFERROR(('Margin Calculator'!$B$6+'Margin Calculator'!$B$7)*'Margin Calculator'!$B$9/(1-'Margin Calculator'!$B$8),0)</f>
-        <v>161.538461538462</v>
-      </c>
-      <c r="J11" s="26" t="str">
+        <v>150</v>
+      </c>
+      <c r="J11" s="27" t="str">
         <f aca="false">IF(D11=0,"–",IF(H11&gt;='Margin Calculator'!$B$8,"Yes","No"))</f>
         <v>Yes</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="25" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="26" t="n">
         <v>40</v>
       </c>
-      <c r="B12" s="26" t="str">
+      <c r="B12" s="27" t="str">
         <f aca="false">IF(AND(A12&gt;='Margin Calculator'!$F$6,A12&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(A12,'Margin Calculator'!$F$6:$F$8,1)),"Out of range")</f>
         <v>Large</v>
       </c>
-      <c r="C12" s="27" t="n">
+      <c r="C12" s="28" t="n">
         <f aca="false">IF(AND(A12&gt;='Margin Calculator'!$F$6,A12&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(A12,'Margin Calculator'!$F$6:$F$8,1)),0)</f>
         <v>169</v>
       </c>
-      <c r="D12" s="27" t="n">
+      <c r="D12" s="28" t="n">
         <f aca="false">A12*C12*'Margin Calculator'!$B$10/12</f>
         <v>29293.3333333333</v>
       </c>
-      <c r="E12" s="27" t="n">
+      <c r="E12" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$6*A12*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
         <v>18200</v>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$7*A12*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
         <v>0</v>
       </c>
-      <c r="G12" s="27" t="n">
+      <c r="G12" s="28" t="n">
         <f aca="false">D12-E12-F12</f>
         <v>11093.3333333333</v>
       </c>
-      <c r="H12" s="28" t="n">
+      <c r="H12" s="29" t="n">
         <f aca="false">IFERROR(G12/D12,0)</f>
         <v>0.378698224852071</v>
       </c>
-      <c r="I12" s="27" t="n">
+      <c r="I12" s="28" t="n">
         <f aca="false">IFERROR(('Margin Calculator'!$B$6+'Margin Calculator'!$B$7)*'Margin Calculator'!$B$9/(1-'Margin Calculator'!$B$8),0)</f>
-        <v>161.538461538462</v>
-      </c>
-      <c r="J12" s="26" t="str">
+        <v>150</v>
+      </c>
+      <c r="J12" s="27" t="str">
         <f aca="false">IF(D12=0,"–",IF(H12&gt;='Margin Calculator'!$B$8,"Yes","No"))</f>
         <v>Yes</v>
       </c>
@@ -1893,896 +1897,896 @@
   <dimension ref="A1:K31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="24" t="s">
+      <c r="A4" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="B4" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="C4" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="D4" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="24" t="s">
+      <c r="E4" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="F4" s="24" t="s">
+      <c r="F4" s="25" t="s">
         <v>69</v>
       </c>
-      <c r="G4" s="24" t="s">
+      <c r="G4" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="H4" s="24" t="s">
+      <c r="H4" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="I4" s="24" t="s">
+      <c r="I4" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="J4" s="24" t="s">
+      <c r="J4" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="K4" s="24" t="s">
+      <c r="K4" s="25" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="29"/>
-      <c r="B5" s="25"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="26" t="str">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="30"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="27" t="str">
         <f aca="false">IF(B5&lt;&gt;"",IF(AND(B5&gt;='Margin Calculator'!$F$6,B5&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B5,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E5" s="27" t="str">
+      <c r="E5" s="28" t="str">
         <f aca="false">IF(B5&lt;&gt;"",IF(AND(B5&gt;='Margin Calculator'!$F$6,B5&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B5,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F5" s="27" t="str">
+      <c r="F5" s="28" t="str">
         <f aca="false">IF(B5&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E5*B5*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E5*B5*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G5" s="27" t="str">
+      <c r="G5" s="28" t="str">
         <f aca="false">IF(B5&lt;&gt;"",IF(C5="",'Margin Calculator'!$B$6,C5)*B5*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H5" s="27" t="str">
+      <c r="H5" s="28" t="str">
         <f aca="false">IF(B5&lt;&gt;"",'Margin Calculator'!$B$7*B5*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I5" s="27" t="str">
+      <c r="I5" s="28" t="str">
         <f aca="false">IF(B5&lt;&gt;"",F5-G5-H5,"")</f>
         <v/>
       </c>
-      <c r="J5" s="28" t="str">
+      <c r="J5" s="29" t="str">
         <f aca="false">IF(B5&lt;&gt;"",IFERROR(I5/F5,0),"")</f>
         <v/>
       </c>
-      <c r="K5" s="26" t="str">
+      <c r="K5" s="27" t="str">
         <f aca="false">IF(B5&lt;&gt;"",IF(E5=0,"Fix hours",IF(J5&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="29"/>
-      <c r="B6" s="25"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="26" t="str">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="30"/>
+      <c r="B6" s="26"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="27" t="str">
         <f aca="false">IF(B6&lt;&gt;"",IF(AND(B6&gt;='Margin Calculator'!$F$6,B6&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B6,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E6" s="27" t="str">
+      <c r="E6" s="28" t="str">
         <f aca="false">IF(B6&lt;&gt;"",IF(AND(B6&gt;='Margin Calculator'!$F$6,B6&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B6,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F6" s="27" t="str">
+      <c r="F6" s="28" t="str">
         <f aca="false">IF(B6&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E6*B6*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E6*B6*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G6" s="27" t="str">
+      <c r="G6" s="28" t="str">
         <f aca="false">IF(B6&lt;&gt;"",IF(C6="",'Margin Calculator'!$B$6,C6)*B6*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H6" s="27" t="str">
+      <c r="H6" s="28" t="str">
         <f aca="false">IF(B6&lt;&gt;"",'Margin Calculator'!$B$7*B6*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I6" s="27" t="str">
+      <c r="I6" s="28" t="str">
         <f aca="false">IF(B6&lt;&gt;"",F6-G6-H6,"")</f>
         <v/>
       </c>
-      <c r="J6" s="28" t="str">
+      <c r="J6" s="29" t="str">
         <f aca="false">IF(B6&lt;&gt;"",IFERROR(I6/F6,0),"")</f>
         <v/>
       </c>
-      <c r="K6" s="26" t="str">
+      <c r="K6" s="27" t="str">
         <f aca="false">IF(B6&lt;&gt;"",IF(E6=0,"Fix hours",IF(J6&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="29"/>
-      <c r="B7" s="25"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="26" t="str">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="30"/>
+      <c r="B7" s="26"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="27" t="str">
         <f aca="false">IF(B7&lt;&gt;"",IF(AND(B7&gt;='Margin Calculator'!$F$6,B7&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B7,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E7" s="27" t="str">
+      <c r="E7" s="28" t="str">
         <f aca="false">IF(B7&lt;&gt;"",IF(AND(B7&gt;='Margin Calculator'!$F$6,B7&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B7,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F7" s="27" t="str">
+      <c r="F7" s="28" t="str">
         <f aca="false">IF(B7&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E7*B7*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E7*B7*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G7" s="27" t="str">
+      <c r="G7" s="28" t="str">
         <f aca="false">IF(B7&lt;&gt;"",IF(C7="",'Margin Calculator'!$B$6,C7)*B7*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H7" s="27" t="str">
+      <c r="H7" s="28" t="str">
         <f aca="false">IF(B7&lt;&gt;"",'Margin Calculator'!$B$7*B7*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I7" s="27" t="str">
+      <c r="I7" s="28" t="str">
         <f aca="false">IF(B7&lt;&gt;"",F7-G7-H7,"")</f>
         <v/>
       </c>
-      <c r="J7" s="28" t="str">
+      <c r="J7" s="29" t="str">
         <f aca="false">IF(B7&lt;&gt;"",IFERROR(I7/F7,0),"")</f>
         <v/>
       </c>
-      <c r="K7" s="26" t="str">
+      <c r="K7" s="27" t="str">
         <f aca="false">IF(B7&lt;&gt;"",IF(E7=0,"Fix hours",IF(J7&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="29"/>
-      <c r="B8" s="25"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="26" t="str">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="30"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="27" t="str">
         <f aca="false">IF(B8&lt;&gt;"",IF(AND(B8&gt;='Margin Calculator'!$F$6,B8&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B8,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E8" s="27" t="str">
+      <c r="E8" s="28" t="str">
         <f aca="false">IF(B8&lt;&gt;"",IF(AND(B8&gt;='Margin Calculator'!$F$6,B8&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B8,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F8" s="27" t="str">
+      <c r="F8" s="28" t="str">
         <f aca="false">IF(B8&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E8*B8*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E8*B8*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G8" s="27" t="str">
+      <c r="G8" s="28" t="str">
         <f aca="false">IF(B8&lt;&gt;"",IF(C8="",'Margin Calculator'!$B$6,C8)*B8*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H8" s="27" t="str">
+      <c r="H8" s="28" t="str">
         <f aca="false">IF(B8&lt;&gt;"",'Margin Calculator'!$B$7*B8*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I8" s="27" t="str">
+      <c r="I8" s="28" t="str">
         <f aca="false">IF(B8&lt;&gt;"",F8-G8-H8,"")</f>
         <v/>
       </c>
-      <c r="J8" s="28" t="str">
+      <c r="J8" s="29" t="str">
         <f aca="false">IF(B8&lt;&gt;"",IFERROR(I8/F8,0),"")</f>
         <v/>
       </c>
-      <c r="K8" s="26" t="str">
+      <c r="K8" s="27" t="str">
         <f aca="false">IF(B8&lt;&gt;"",IF(E8=0,"Fix hours",IF(J8&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="29"/>
-      <c r="B9" s="25"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="26" t="str">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="30"/>
+      <c r="B9" s="26"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="27" t="str">
         <f aca="false">IF(B9&lt;&gt;"",IF(AND(B9&gt;='Margin Calculator'!$F$6,B9&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B9,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E9" s="27" t="str">
+      <c r="E9" s="28" t="str">
         <f aca="false">IF(B9&lt;&gt;"",IF(AND(B9&gt;='Margin Calculator'!$F$6,B9&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B9,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F9" s="27" t="str">
+      <c r="F9" s="28" t="str">
         <f aca="false">IF(B9&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E9*B9*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E9*B9*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G9" s="27" t="str">
+      <c r="G9" s="28" t="str">
         <f aca="false">IF(B9&lt;&gt;"",IF(C9="",'Margin Calculator'!$B$6,C9)*B9*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H9" s="27" t="str">
+      <c r="H9" s="28" t="str">
         <f aca="false">IF(B9&lt;&gt;"",'Margin Calculator'!$B$7*B9*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I9" s="27" t="str">
+      <c r="I9" s="28" t="str">
         <f aca="false">IF(B9&lt;&gt;"",F9-G9-H9,"")</f>
         <v/>
       </c>
-      <c r="J9" s="28" t="str">
+      <c r="J9" s="29" t="str">
         <f aca="false">IF(B9&lt;&gt;"",IFERROR(I9/F9,0),"")</f>
         <v/>
       </c>
-      <c r="K9" s="26" t="str">
+      <c r="K9" s="27" t="str">
         <f aca="false">IF(B9&lt;&gt;"",IF(E9=0,"Fix hours",IF(J9&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="29"/>
-      <c r="B10" s="25"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="26" t="str">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="30"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="27" t="str">
         <f aca="false">IF(B10&lt;&gt;"",IF(AND(B10&gt;='Margin Calculator'!$F$6,B10&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B10,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E10" s="27" t="str">
+      <c r="E10" s="28" t="str">
         <f aca="false">IF(B10&lt;&gt;"",IF(AND(B10&gt;='Margin Calculator'!$F$6,B10&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B10,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F10" s="27" t="str">
+      <c r="F10" s="28" t="str">
         <f aca="false">IF(B10&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E10*B10*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E10*B10*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G10" s="27" t="str">
+      <c r="G10" s="28" t="str">
         <f aca="false">IF(B10&lt;&gt;"",IF(C10="",'Margin Calculator'!$B$6,C10)*B10*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H10" s="27" t="str">
+      <c r="H10" s="28" t="str">
         <f aca="false">IF(B10&lt;&gt;"",'Margin Calculator'!$B$7*B10*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I10" s="27" t="str">
+      <c r="I10" s="28" t="str">
         <f aca="false">IF(B10&lt;&gt;"",F10-G10-H10,"")</f>
         <v/>
       </c>
-      <c r="J10" s="28" t="str">
+      <c r="J10" s="29" t="str">
         <f aca="false">IF(B10&lt;&gt;"",IFERROR(I10/F10,0),"")</f>
         <v/>
       </c>
-      <c r="K10" s="26" t="str">
+      <c r="K10" s="27" t="str">
         <f aca="false">IF(B10&lt;&gt;"",IF(E10=0,"Fix hours",IF(J10&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="29"/>
-      <c r="B11" s="25"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="26" t="str">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="30"/>
+      <c r="B11" s="26"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="27" t="str">
         <f aca="false">IF(B11&lt;&gt;"",IF(AND(B11&gt;='Margin Calculator'!$F$6,B11&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B11,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E11" s="27" t="str">
+      <c r="E11" s="28" t="str">
         <f aca="false">IF(B11&lt;&gt;"",IF(AND(B11&gt;='Margin Calculator'!$F$6,B11&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B11,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F11" s="27" t="str">
+      <c r="F11" s="28" t="str">
         <f aca="false">IF(B11&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E11*B11*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E11*B11*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G11" s="27" t="str">
+      <c r="G11" s="28" t="str">
         <f aca="false">IF(B11&lt;&gt;"",IF(C11="",'Margin Calculator'!$B$6,C11)*B11*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H11" s="27" t="str">
+      <c r="H11" s="28" t="str">
         <f aca="false">IF(B11&lt;&gt;"",'Margin Calculator'!$B$7*B11*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I11" s="27" t="str">
+      <c r="I11" s="28" t="str">
         <f aca="false">IF(B11&lt;&gt;"",F11-G11-H11,"")</f>
         <v/>
       </c>
-      <c r="J11" s="28" t="str">
+      <c r="J11" s="29" t="str">
         <f aca="false">IF(B11&lt;&gt;"",IFERROR(I11/F11,0),"")</f>
         <v/>
       </c>
-      <c r="K11" s="26" t="str">
+      <c r="K11" s="27" t="str">
         <f aca="false">IF(B11&lt;&gt;"",IF(E11=0,"Fix hours",IF(J11&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="29"/>
-      <c r="B12" s="25"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="26" t="str">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="30"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="27" t="str">
         <f aca="false">IF(B12&lt;&gt;"",IF(AND(B12&gt;='Margin Calculator'!$F$6,B12&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B12,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E12" s="27" t="str">
+      <c r="E12" s="28" t="str">
         <f aca="false">IF(B12&lt;&gt;"",IF(AND(B12&gt;='Margin Calculator'!$F$6,B12&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B12,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F12" s="27" t="str">
+      <c r="F12" s="28" t="str">
         <f aca="false">IF(B12&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E12*B12*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E12*B12*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G12" s="27" t="str">
+      <c r="G12" s="28" t="str">
         <f aca="false">IF(B12&lt;&gt;"",IF(C12="",'Margin Calculator'!$B$6,C12)*B12*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H12" s="27" t="str">
+      <c r="H12" s="28" t="str">
         <f aca="false">IF(B12&lt;&gt;"",'Margin Calculator'!$B$7*B12*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I12" s="27" t="str">
+      <c r="I12" s="28" t="str">
         <f aca="false">IF(B12&lt;&gt;"",F12-G12-H12,"")</f>
         <v/>
       </c>
-      <c r="J12" s="28" t="str">
+      <c r="J12" s="29" t="str">
         <f aca="false">IF(B12&lt;&gt;"",IFERROR(I12/F12,0),"")</f>
         <v/>
       </c>
-      <c r="K12" s="26" t="str">
+      <c r="K12" s="27" t="str">
         <f aca="false">IF(B12&lt;&gt;"",IF(E12=0,"Fix hours",IF(J12&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="29"/>
-      <c r="B13" s="25"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="26" t="str">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="30"/>
+      <c r="B13" s="26"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="27" t="str">
         <f aca="false">IF(B13&lt;&gt;"",IF(AND(B13&gt;='Margin Calculator'!$F$6,B13&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B13,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E13" s="27" t="str">
+      <c r="E13" s="28" t="str">
         <f aca="false">IF(B13&lt;&gt;"",IF(AND(B13&gt;='Margin Calculator'!$F$6,B13&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B13,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F13" s="27" t="str">
+      <c r="F13" s="28" t="str">
         <f aca="false">IF(B13&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E13*B13*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E13*B13*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G13" s="27" t="str">
+      <c r="G13" s="28" t="str">
         <f aca="false">IF(B13&lt;&gt;"",IF(C13="",'Margin Calculator'!$B$6,C13)*B13*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H13" s="27" t="str">
+      <c r="H13" s="28" t="str">
         <f aca="false">IF(B13&lt;&gt;"",'Margin Calculator'!$B$7*B13*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I13" s="27" t="str">
+      <c r="I13" s="28" t="str">
         <f aca="false">IF(B13&lt;&gt;"",F13-G13-H13,"")</f>
         <v/>
       </c>
-      <c r="J13" s="28" t="str">
+      <c r="J13" s="29" t="str">
         <f aca="false">IF(B13&lt;&gt;"",IFERROR(I13/F13,0),"")</f>
         <v/>
       </c>
-      <c r="K13" s="26" t="str">
+      <c r="K13" s="27" t="str">
         <f aca="false">IF(B13&lt;&gt;"",IF(E13=0,"Fix hours",IF(J13&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="29"/>
-      <c r="B14" s="25"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="26" t="str">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="30"/>
+      <c r="B14" s="26"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="27" t="str">
         <f aca="false">IF(B14&lt;&gt;"",IF(AND(B14&gt;='Margin Calculator'!$F$6,B14&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B14,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E14" s="27" t="str">
+      <c r="E14" s="28" t="str">
         <f aca="false">IF(B14&lt;&gt;"",IF(AND(B14&gt;='Margin Calculator'!$F$6,B14&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B14,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F14" s="27" t="str">
+      <c r="F14" s="28" t="str">
         <f aca="false">IF(B14&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E14*B14*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E14*B14*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G14" s="27" t="str">
+      <c r="G14" s="28" t="str">
         <f aca="false">IF(B14&lt;&gt;"",IF(C14="",'Margin Calculator'!$B$6,C14)*B14*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H14" s="27" t="str">
+      <c r="H14" s="28" t="str">
         <f aca="false">IF(B14&lt;&gt;"",'Margin Calculator'!$B$7*B14*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I14" s="27" t="str">
+      <c r="I14" s="28" t="str">
         <f aca="false">IF(B14&lt;&gt;"",F14-G14-H14,"")</f>
         <v/>
       </c>
-      <c r="J14" s="28" t="str">
+      <c r="J14" s="29" t="str">
         <f aca="false">IF(B14&lt;&gt;"",IFERROR(I14/F14,0),"")</f>
         <v/>
       </c>
-      <c r="K14" s="26" t="str">
+      <c r="K14" s="27" t="str">
         <f aca="false">IF(B14&lt;&gt;"",IF(E14=0,"Fix hours",IF(J14&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="29"/>
-      <c r="B15" s="25"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="26" t="str">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="30"/>
+      <c r="B15" s="26"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="27" t="str">
         <f aca="false">IF(B15&lt;&gt;"",IF(AND(B15&gt;='Margin Calculator'!$F$6,B15&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B15,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E15" s="27" t="str">
+      <c r="E15" s="28" t="str">
         <f aca="false">IF(B15&lt;&gt;"",IF(AND(B15&gt;='Margin Calculator'!$F$6,B15&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B15,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F15" s="27" t="str">
+      <c r="F15" s="28" t="str">
         <f aca="false">IF(B15&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E15*B15*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E15*B15*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G15" s="27" t="str">
+      <c r="G15" s="28" t="str">
         <f aca="false">IF(B15&lt;&gt;"",IF(C15="",'Margin Calculator'!$B$6,C15)*B15*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H15" s="27" t="str">
+      <c r="H15" s="28" t="str">
         <f aca="false">IF(B15&lt;&gt;"",'Margin Calculator'!$B$7*B15*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I15" s="27" t="str">
+      <c r="I15" s="28" t="str">
         <f aca="false">IF(B15&lt;&gt;"",F15-G15-H15,"")</f>
         <v/>
       </c>
-      <c r="J15" s="28" t="str">
+      <c r="J15" s="29" t="str">
         <f aca="false">IF(B15&lt;&gt;"",IFERROR(I15/F15,0),"")</f>
         <v/>
       </c>
-      <c r="K15" s="26" t="str">
+      <c r="K15" s="27" t="str">
         <f aca="false">IF(B15&lt;&gt;"",IF(E15=0,"Fix hours",IF(J15&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="29"/>
-      <c r="B16" s="25"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="26" t="str">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="30"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="27" t="str">
         <f aca="false">IF(B16&lt;&gt;"",IF(AND(B16&gt;='Margin Calculator'!$F$6,B16&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B16,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E16" s="27" t="str">
+      <c r="E16" s="28" t="str">
         <f aca="false">IF(B16&lt;&gt;"",IF(AND(B16&gt;='Margin Calculator'!$F$6,B16&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B16,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F16" s="27" t="str">
+      <c r="F16" s="28" t="str">
         <f aca="false">IF(B16&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E16*B16*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E16*B16*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G16" s="27" t="str">
+      <c r="G16" s="28" t="str">
         <f aca="false">IF(B16&lt;&gt;"",IF(C16="",'Margin Calculator'!$B$6,C16)*B16*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H16" s="27" t="str">
+      <c r="H16" s="28" t="str">
         <f aca="false">IF(B16&lt;&gt;"",'Margin Calculator'!$B$7*B16*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I16" s="27" t="str">
+      <c r="I16" s="28" t="str">
         <f aca="false">IF(B16&lt;&gt;"",F16-G16-H16,"")</f>
         <v/>
       </c>
-      <c r="J16" s="28" t="str">
+      <c r="J16" s="29" t="str">
         <f aca="false">IF(B16&lt;&gt;"",IFERROR(I16/F16,0),"")</f>
         <v/>
       </c>
-      <c r="K16" s="26" t="str">
+      <c r="K16" s="27" t="str">
         <f aca="false">IF(B16&lt;&gt;"",IF(E16=0,"Fix hours",IF(J16&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="29"/>
-      <c r="B17" s="25"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="26" t="str">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="30"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="27" t="str">
         <f aca="false">IF(B17&lt;&gt;"",IF(AND(B17&gt;='Margin Calculator'!$F$6,B17&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B17,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E17" s="27" t="str">
+      <c r="E17" s="28" t="str">
         <f aca="false">IF(B17&lt;&gt;"",IF(AND(B17&gt;='Margin Calculator'!$F$6,B17&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B17,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F17" s="27" t="str">
+      <c r="F17" s="28" t="str">
         <f aca="false">IF(B17&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E17*B17*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E17*B17*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G17" s="27" t="str">
+      <c r="G17" s="28" t="str">
         <f aca="false">IF(B17&lt;&gt;"",IF(C17="",'Margin Calculator'!$B$6,C17)*B17*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H17" s="27" t="str">
+      <c r="H17" s="28" t="str">
         <f aca="false">IF(B17&lt;&gt;"",'Margin Calculator'!$B$7*B17*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I17" s="27" t="str">
+      <c r="I17" s="28" t="str">
         <f aca="false">IF(B17&lt;&gt;"",F17-G17-H17,"")</f>
         <v/>
       </c>
-      <c r="J17" s="28" t="str">
+      <c r="J17" s="29" t="str">
         <f aca="false">IF(B17&lt;&gt;"",IFERROR(I17/F17,0),"")</f>
         <v/>
       </c>
-      <c r="K17" s="26" t="str">
+      <c r="K17" s="27" t="str">
         <f aca="false">IF(B17&lt;&gt;"",IF(E17=0,"Fix hours",IF(J17&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="29"/>
-      <c r="B18" s="25"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="26" t="str">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="30"/>
+      <c r="B18" s="26"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="27" t="str">
         <f aca="false">IF(B18&lt;&gt;"",IF(AND(B18&gt;='Margin Calculator'!$F$6,B18&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B18,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E18" s="27" t="str">
+      <c r="E18" s="28" t="str">
         <f aca="false">IF(B18&lt;&gt;"",IF(AND(B18&gt;='Margin Calculator'!$F$6,B18&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B18,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F18" s="27" t="str">
+      <c r="F18" s="28" t="str">
         <f aca="false">IF(B18&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E18*B18*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E18*B18*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G18" s="27" t="str">
+      <c r="G18" s="28" t="str">
         <f aca="false">IF(B18&lt;&gt;"",IF(C18="",'Margin Calculator'!$B$6,C18)*B18*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H18" s="27" t="str">
+      <c r="H18" s="28" t="str">
         <f aca="false">IF(B18&lt;&gt;"",'Margin Calculator'!$B$7*B18*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I18" s="27" t="str">
+      <c r="I18" s="28" t="str">
         <f aca="false">IF(B18&lt;&gt;"",F18-G18-H18,"")</f>
         <v/>
       </c>
-      <c r="J18" s="28" t="str">
+      <c r="J18" s="29" t="str">
         <f aca="false">IF(B18&lt;&gt;"",IFERROR(I18/F18,0),"")</f>
         <v/>
       </c>
-      <c r="K18" s="26" t="str">
+      <c r="K18" s="27" t="str">
         <f aca="false">IF(B18&lt;&gt;"",IF(E18=0,"Fix hours",IF(J18&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="29"/>
-      <c r="B19" s="25"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="26" t="str">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="30"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="27" t="str">
         <f aca="false">IF(B19&lt;&gt;"",IF(AND(B19&gt;='Margin Calculator'!$F$6,B19&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B19,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E19" s="27" t="str">
+      <c r="E19" s="28" t="str">
         <f aca="false">IF(B19&lt;&gt;"",IF(AND(B19&gt;='Margin Calculator'!$F$6,B19&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B19,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F19" s="27" t="str">
+      <c r="F19" s="28" t="str">
         <f aca="false">IF(B19&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E19*B19*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E19*B19*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G19" s="27" t="str">
+      <c r="G19" s="28" t="str">
         <f aca="false">IF(B19&lt;&gt;"",IF(C19="",'Margin Calculator'!$B$6,C19)*B19*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H19" s="27" t="str">
+      <c r="H19" s="28" t="str">
         <f aca="false">IF(B19&lt;&gt;"",'Margin Calculator'!$B$7*B19*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I19" s="27" t="str">
+      <c r="I19" s="28" t="str">
         <f aca="false">IF(B19&lt;&gt;"",F19-G19-H19,"")</f>
         <v/>
       </c>
-      <c r="J19" s="28" t="str">
+      <c r="J19" s="29" t="str">
         <f aca="false">IF(B19&lt;&gt;"",IFERROR(I19/F19,0),"")</f>
         <v/>
       </c>
-      <c r="K19" s="26" t="str">
+      <c r="K19" s="27" t="str">
         <f aca="false">IF(B19&lt;&gt;"",IF(E19=0,"Fix hours",IF(J19&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="29"/>
-      <c r="B20" s="25"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="26" t="str">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="30"/>
+      <c r="B20" s="26"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="27" t="str">
         <f aca="false">IF(B20&lt;&gt;"",IF(AND(B20&gt;='Margin Calculator'!$F$6,B20&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B20,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E20" s="27" t="str">
+      <c r="E20" s="28" t="str">
         <f aca="false">IF(B20&lt;&gt;"",IF(AND(B20&gt;='Margin Calculator'!$F$6,B20&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B20,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F20" s="27" t="str">
+      <c r="F20" s="28" t="str">
         <f aca="false">IF(B20&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E20*B20*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E20*B20*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G20" s="27" t="str">
+      <c r="G20" s="28" t="str">
         <f aca="false">IF(B20&lt;&gt;"",IF(C20="",'Margin Calculator'!$B$6,C20)*B20*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H20" s="27" t="str">
+      <c r="H20" s="28" t="str">
         <f aca="false">IF(B20&lt;&gt;"",'Margin Calculator'!$B$7*B20*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I20" s="27" t="str">
+      <c r="I20" s="28" t="str">
         <f aca="false">IF(B20&lt;&gt;"",F20-G20-H20,"")</f>
         <v/>
       </c>
-      <c r="J20" s="28" t="str">
+      <c r="J20" s="29" t="str">
         <f aca="false">IF(B20&lt;&gt;"",IFERROR(I20/F20,0),"")</f>
         <v/>
       </c>
-      <c r="K20" s="26" t="str">
+      <c r="K20" s="27" t="str">
         <f aca="false">IF(B20&lt;&gt;"",IF(E20=0,"Fix hours",IF(J20&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="29"/>
-      <c r="B21" s="25"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="26" t="str">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="30"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="27" t="str">
         <f aca="false">IF(B21&lt;&gt;"",IF(AND(B21&gt;='Margin Calculator'!$F$6,B21&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B21,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E21" s="27" t="str">
+      <c r="E21" s="28" t="str">
         <f aca="false">IF(B21&lt;&gt;"",IF(AND(B21&gt;='Margin Calculator'!$F$6,B21&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B21,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F21" s="27" t="str">
+      <c r="F21" s="28" t="str">
         <f aca="false">IF(B21&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E21*B21*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E21*B21*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G21" s="27" t="str">
+      <c r="G21" s="28" t="str">
         <f aca="false">IF(B21&lt;&gt;"",IF(C21="",'Margin Calculator'!$B$6,C21)*B21*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H21" s="27" t="str">
+      <c r="H21" s="28" t="str">
         <f aca="false">IF(B21&lt;&gt;"",'Margin Calculator'!$B$7*B21*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I21" s="27" t="str">
+      <c r="I21" s="28" t="str">
         <f aca="false">IF(B21&lt;&gt;"",F21-G21-H21,"")</f>
         <v/>
       </c>
-      <c r="J21" s="28" t="str">
+      <c r="J21" s="29" t="str">
         <f aca="false">IF(B21&lt;&gt;"",IFERROR(I21/F21,0),"")</f>
         <v/>
       </c>
-      <c r="K21" s="26" t="str">
+      <c r="K21" s="27" t="str">
         <f aca="false">IF(B21&lt;&gt;"",IF(E21=0,"Fix hours",IF(J21&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="29"/>
-      <c r="B22" s="25"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="26" t="str">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="30"/>
+      <c r="B22" s="26"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="27" t="str">
         <f aca="false">IF(B22&lt;&gt;"",IF(AND(B22&gt;='Margin Calculator'!$F$6,B22&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B22,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E22" s="27" t="str">
+      <c r="E22" s="28" t="str">
         <f aca="false">IF(B22&lt;&gt;"",IF(AND(B22&gt;='Margin Calculator'!$F$6,B22&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B22,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F22" s="27" t="str">
+      <c r="F22" s="28" t="str">
         <f aca="false">IF(B22&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E22*B22*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E22*B22*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G22" s="27" t="str">
+      <c r="G22" s="28" t="str">
         <f aca="false">IF(B22&lt;&gt;"",IF(C22="",'Margin Calculator'!$B$6,C22)*B22*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H22" s="27" t="str">
+      <c r="H22" s="28" t="str">
         <f aca="false">IF(B22&lt;&gt;"",'Margin Calculator'!$B$7*B22*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I22" s="27" t="str">
+      <c r="I22" s="28" t="str">
         <f aca="false">IF(B22&lt;&gt;"",F22-G22-H22,"")</f>
         <v/>
       </c>
-      <c r="J22" s="28" t="str">
+      <c r="J22" s="29" t="str">
         <f aca="false">IF(B22&lt;&gt;"",IFERROR(I22/F22,0),"")</f>
         <v/>
       </c>
-      <c r="K22" s="26" t="str">
+      <c r="K22" s="27" t="str">
         <f aca="false">IF(B22&lt;&gt;"",IF(E22=0,"Fix hours",IF(J22&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="29"/>
-      <c r="B23" s="25"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="26" t="str">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="30"/>
+      <c r="B23" s="26"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="27" t="str">
         <f aca="false">IF(B23&lt;&gt;"",IF(AND(B23&gt;='Margin Calculator'!$F$6,B23&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B23,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E23" s="27" t="str">
+      <c r="E23" s="28" t="str">
         <f aca="false">IF(B23&lt;&gt;"",IF(AND(B23&gt;='Margin Calculator'!$F$6,B23&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B23,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F23" s="27" t="str">
+      <c r="F23" s="28" t="str">
         <f aca="false">IF(B23&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E23*B23*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E23*B23*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G23" s="27" t="str">
+      <c r="G23" s="28" t="str">
         <f aca="false">IF(B23&lt;&gt;"",IF(C23="",'Margin Calculator'!$B$6,C23)*B23*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H23" s="27" t="str">
+      <c r="H23" s="28" t="str">
         <f aca="false">IF(B23&lt;&gt;"",'Margin Calculator'!$B$7*B23*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I23" s="27" t="str">
+      <c r="I23" s="28" t="str">
         <f aca="false">IF(B23&lt;&gt;"",F23-G23-H23,"")</f>
         <v/>
       </c>
-      <c r="J23" s="28" t="str">
+      <c r="J23" s="29" t="str">
         <f aca="false">IF(B23&lt;&gt;"",IFERROR(I23/F23,0),"")</f>
         <v/>
       </c>
-      <c r="K23" s="26" t="str">
+      <c r="K23" s="27" t="str">
         <f aca="false">IF(B23&lt;&gt;"",IF(E23=0,"Fix hours",IF(J23&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="29"/>
-      <c r="B24" s="25"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="26" t="str">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="30"/>
+      <c r="B24" s="26"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="27" t="str">
         <f aca="false">IF(B24&lt;&gt;"",IF(AND(B24&gt;='Margin Calculator'!$F$6,B24&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(B24,'Margin Calculator'!$F$6:$F$8,1)),"Out of range"),"")</f>
         <v/>
       </c>
-      <c r="E24" s="27" t="str">
+      <c r="E24" s="28" t="str">
         <f aca="false">IF(B24&lt;&gt;"",IF(AND(B24&gt;='Margin Calculator'!$F$6,B24&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(B24,'Margin Calculator'!$F$6:$F$8,1)),0),"")</f>
         <v/>
       </c>
-      <c r="F24" s="27" t="str">
+      <c r="F24" s="28" t="str">
         <f aca="false">IF(B24&lt;&gt;"",IF('Margin Calculator'!$B$11&gt;0,CEILING(E24*B24*'Margin Calculator'!$B$10/12,'Margin Calculator'!$B$11),E24*B24*'Margin Calculator'!$B$10/12),"")</f>
         <v/>
       </c>
-      <c r="G24" s="27" t="str">
+      <c r="G24" s="28" t="str">
         <f aca="false">IF(B24&lt;&gt;"",IF(C24="",'Margin Calculator'!$B$6,C24)*B24*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="H24" s="27" t="str">
+      <c r="H24" s="28" t="str">
         <f aca="false">IF(B24&lt;&gt;"",'Margin Calculator'!$B$7*B24*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12,"")</f>
         <v/>
       </c>
-      <c r="I24" s="27" t="str">
+      <c r="I24" s="28" t="str">
         <f aca="false">IF(B24&lt;&gt;"",F24-G24-H24,"")</f>
         <v/>
       </c>
-      <c r="J24" s="28" t="str">
+      <c r="J24" s="29" t="str">
         <f aca="false">IF(B24&lt;&gt;"",IFERROR(I24/F24,0),"")</f>
         <v/>
       </c>
-      <c r="K24" s="26" t="str">
+      <c r="K24" s="27" t="str">
         <f aca="false">IF(B24&lt;&gt;"",IF(E24=0,"Fix hours",IF(J24&gt;='Margin Calculator'!$B$8,"Yes","No")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="30" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="31" t="s">
         <v>71</v>
       </c>
-      <c r="B26" s="31" t="n">
+      <c r="B26" s="32" t="n">
         <f aca="false">SUM(B5:B24)</f>
         <v>0</v>
       </c>
-      <c r="C26" s="32"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32"/>
-      <c r="F26" s="33" t="n">
+      <c r="C26" s="33"/>
+      <c r="D26" s="33"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="34" t="n">
         <f aca="false">SUM(F5:F24)</f>
         <v>0</v>
       </c>
-      <c r="G26" s="33" t="n">
+      <c r="G26" s="34" t="n">
         <f aca="false">SUM(G5:G24)</f>
         <v>0</v>
       </c>
-      <c r="H26" s="33" t="n">
+      <c r="H26" s="34" t="n">
         <f aca="false">SUM(H5:H24)</f>
         <v>0</v>
       </c>
-      <c r="I26" s="33" t="n">
+      <c r="I26" s="34" t="n">
         <f aca="false">SUM(I5:I24)</f>
         <v>0</v>
       </c>
-      <c r="J26" s="34" t="n">
+      <c r="J26" s="35" t="n">
         <f aca="false">IFERROR(I26/F26,0)</f>
         <v>0</v>
       </c>
-      <c r="K26" s="32"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="35" t="s">
+      <c r="K26" s="33"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="36" t="s">
         <v>72</v>
       </c>
-      <c r="B28" s="35"/>
-      <c r="C28" s="35"/>
-      <c r="D28" s="36" t="n">
+      <c r="B28" s="36"/>
+      <c r="C28" s="36"/>
+      <c r="D28" s="37" t="n">
         <f aca="false">COUNTA(A5:A24)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="35" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="36" t="s">
         <v>73</v>
       </c>
-      <c r="B29" s="35"/>
-      <c r="C29" s="35"/>
-      <c r="D29" s="37" t="n">
+      <c r="B29" s="36"/>
+      <c r="C29" s="36"/>
+      <c r="D29" s="38" t="n">
         <f aca="false">F26*12</f>
         <v>0</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="35" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="B30" s="35"/>
-      <c r="C30" s="35"/>
-      <c r="D30" s="37" t="n">
+      <c r="B30" s="36"/>
+      <c r="C30" s="36"/>
+      <c r="D30" s="38" t="n">
         <f aca="false">I26*12</f>
         <v>0</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="35" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="36" t="s">
         <v>74</v>
       </c>
-      <c r="B31" s="35"/>
-      <c r="C31" s="35"/>
-      <c r="D31" s="38" t="n">
+      <c r="B31" s="36"/>
+      <c r="C31" s="36"/>
+      <c r="D31" s="39" t="n">
         <f aca="false">B26*'Margin Calculator'!$B$9/40</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Fix tier price dips, new tier names, backup/restore, contract term, blended team
- Default tiers: Lite Engagement $189 / Part-Time $180 / Full-Time $174 (no price dips);
  saved browser data is moved to the new names and rates once
- Backup & restore: download or copy a backup, restore from file or pasted text (with Undo)
- Contract term: monthly, 6 or 12 months with editable discount; flows into quote,
  margin, lowest rate, contract value and P&L
- Blended team: roles with % of hours and $/hr; drives 1099 cost and P&L rows
- Excel: tier names and rates updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GHAGAmwRkNyFBmFrnvVcew
</commit_message>
<xml_diff>
--- a/Catalyst_IQ_Labs_AMS_Margin_Calculator_Weekly_-_V2.xlsx
+++ b/Catalyst_IQ_Labs_AMS_Margin_Calculator_Weekly_-_V2.xlsx
@@ -109,7 +109,7 @@
     <t xml:space="preserve">What you pay the contractor per hour worked.</t>
   </si>
   <si>
-    <t xml:space="preserve">Small</t>
+    <t xml:space="preserve">Lite Engagement</t>
   </si>
   <si>
     <t xml:space="preserve">Overhead allocation ($/hr)</t>
@@ -118,7 +118,7 @@
     <t xml:space="preserve">Your share of tools, insurance, admin, etc. per hour delivered. Leave $0 to ignore.</t>
   </si>
   <si>
-    <t xml:space="preserve">Mid</t>
+    <t xml:space="preserve">Part-Time</t>
   </si>
   <si>
     <t xml:space="preserve">Target contribution margin</t>
@@ -127,7 +127,7 @@
     <t xml:space="preserve">The minimum margin you want to keep after consultant cost and overhead.</t>
   </si>
   <si>
-    <t xml:space="preserve">Large</t>
+    <t xml:space="preserve">Full-Time</t>
   </si>
   <si>
     <t xml:space="preserve">Hours actually delivered (% of contracted)</t>
@@ -952,7 +952,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="14"/>
   </cols>
@@ -1060,7 +1060,7 @@
         <v>29</v>
       </c>
       <c r="H7" s="12" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1083,7 +1083,7 @@
         <v>40</v>
       </c>
       <c r="H8" s="12" t="n">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="B14" s="18" t="str">
         <f aca="false">IF(AND($B$5&gt;=$F$6,$B$5&lt;=$G$8),INDEX($E$6:$E$8,MATCH($B$5,$F$6:$F$8,1)),"Out of range")</f>
-        <v>Small</v>
+        <v>Lite Engagement</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="B5" s="27" t="str">
         <f aca="false">IF(AND(A5&gt;='Margin Calculator'!$F$6,A5&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(A5,'Margin Calculator'!$F$6:$F$8,1)),"Out of range")</f>
-        <v>Small</v>
+        <v>Lite Engagement</v>
       </c>
       <c r="C5" s="28" t="n">
         <f aca="false">IF(AND(A5&gt;='Margin Calculator'!$F$6,A5&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(A5,'Margin Calculator'!$F$6:$F$8,1)),0)</f>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="B6" s="27" t="str">
         <f aca="false">IF(AND(A6&gt;='Margin Calculator'!$F$6,A6&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(A6,'Margin Calculator'!$F$6:$F$8,1)),"Out of range")</f>
-        <v>Small</v>
+        <v>Lite Engagement</v>
       </c>
       <c r="C6" s="28" t="n">
         <f aca="false">IF(AND(A6&gt;='Margin Calculator'!$F$6,A6&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(A6,'Margin Calculator'!$F$6:$F$8,1)),0)</f>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="B7" s="27" t="str">
         <f aca="false">IF(AND(A7&gt;='Margin Calculator'!$F$6,A7&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(A7,'Margin Calculator'!$F$6:$F$8,1)),"Out of range")</f>
-        <v>Small</v>
+        <v>Lite Engagement</v>
       </c>
       <c r="C7" s="28" t="n">
         <f aca="false">IF(AND(A7&gt;='Margin Calculator'!$F$6,A7&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(A7,'Margin Calculator'!$F$6:$F$8,1)),0)</f>
@@ -1650,7 +1650,7 @@
       </c>
       <c r="B8" s="27" t="str">
         <f aca="false">IF(AND(A8&gt;='Margin Calculator'!$F$6,A8&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(A8,'Margin Calculator'!$F$6:$F$8,1)),"Out of range")</f>
-        <v>Small</v>
+        <v>Lite Engagement</v>
       </c>
       <c r="C8" s="28" t="n">
         <f aca="false">IF(AND(A8&gt;='Margin Calculator'!$F$6,A8&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(A8,'Margin Calculator'!$F$6:$F$8,1)),0)</f>
@@ -1691,15 +1691,15 @@
       </c>
       <c r="B9" s="27" t="str">
         <f aca="false">IF(AND(A9&gt;='Margin Calculator'!$F$6,A9&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(A9,'Margin Calculator'!$F$6:$F$8,1)),"Out of range")</f>
-        <v>Mid</v>
+        <v>Part-Time</v>
       </c>
       <c r="C9" s="28" t="n">
         <f aca="false">IF(AND(A9&gt;='Margin Calculator'!$F$6,A9&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(A9,'Margin Calculator'!$F$6:$F$8,1)),0)</f>
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D9" s="28" t="n">
         <f aca="false">A9*C9*'Margin Calculator'!$B$10/12</f>
-        <v>19391.6666666667</v>
+        <v>19500</v>
       </c>
       <c r="E9" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$6*A9*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
@@ -1711,11 +1711,11 @@
       </c>
       <c r="G9" s="28" t="n">
         <f aca="false">D9-E9-F9</f>
-        <v>8016.66666666667</v>
+        <v>8125</v>
       </c>
       <c r="H9" s="29" t="n">
         <f aca="false">IFERROR(G9/D9,0)</f>
-        <v>0.41340782122905</v>
+        <v>0.416666666666667</v>
       </c>
       <c r="I9" s="28" t="n">
         <f aca="false">IFERROR(('Margin Calculator'!$B$6+'Margin Calculator'!$B$7)*'Margin Calculator'!$B$9/(1-'Margin Calculator'!$B$8),0)</f>
@@ -1732,15 +1732,15 @@
       </c>
       <c r="B10" s="27" t="str">
         <f aca="false">IF(AND(A10&gt;='Margin Calculator'!$F$6,A10&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(A10,'Margin Calculator'!$F$6:$F$8,1)),"Out of range")</f>
-        <v>Large</v>
+        <v>Full-Time</v>
       </c>
       <c r="C10" s="28" t="n">
         <f aca="false">IF(AND(A10&gt;='Margin Calculator'!$F$6,A10&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(A10,'Margin Calculator'!$F$6:$F$8,1)),0)</f>
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D10" s="28" t="n">
         <f aca="false">A10*C10*'Margin Calculator'!$B$10/12</f>
-        <v>21970</v>
+        <v>22620</v>
       </c>
       <c r="E10" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$6*A10*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
@@ -1752,11 +1752,11 @@
       </c>
       <c r="G10" s="28" t="n">
         <f aca="false">D10-E10-F10</f>
-        <v>8320</v>
+        <v>8970</v>
       </c>
       <c r="H10" s="29" t="n">
         <f aca="false">IFERROR(G10/D10,0)</f>
-        <v>0.378698224852071</v>
+        <v>0.396551724137931</v>
       </c>
       <c r="I10" s="28" t="n">
         <f aca="false">IFERROR(('Margin Calculator'!$B$6+'Margin Calculator'!$B$7)*'Margin Calculator'!$B$9/(1-'Margin Calculator'!$B$8),0)</f>
@@ -1773,15 +1773,15 @@
       </c>
       <c r="B11" s="27" t="str">
         <f aca="false">IF(AND(A11&gt;='Margin Calculator'!$F$6,A11&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(A11,'Margin Calculator'!$F$6:$F$8,1)),"Out of range")</f>
-        <v>Large</v>
+        <v>Full-Time</v>
       </c>
       <c r="C11" s="28" t="n">
         <f aca="false">IF(AND(A11&gt;='Margin Calculator'!$F$6,A11&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(A11,'Margin Calculator'!$F$6:$F$8,1)),0)</f>
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D11" s="28" t="n">
         <f aca="false">A11*C11*'Margin Calculator'!$B$10/12</f>
-        <v>25631.6666666667</v>
+        <v>26390</v>
       </c>
       <c r="E11" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$6*A11*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
@@ -1793,11 +1793,11 @@
       </c>
       <c r="G11" s="28" t="n">
         <f aca="false">D11-E11-F11</f>
-        <v>9706.66666666667</v>
+        <v>10465</v>
       </c>
       <c r="H11" s="29" t="n">
         <f aca="false">IFERROR(G11/D11,0)</f>
-        <v>0.378698224852071</v>
+        <v>0.396551724137931</v>
       </c>
       <c r="I11" s="28" t="n">
         <f aca="false">IFERROR(('Margin Calculator'!$B$6+'Margin Calculator'!$B$7)*'Margin Calculator'!$B$9/(1-'Margin Calculator'!$B$8),0)</f>
@@ -1814,15 +1814,15 @@
       </c>
       <c r="B12" s="27" t="str">
         <f aca="false">IF(AND(A12&gt;='Margin Calculator'!$F$6,A12&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$E$6:$E$8,MATCH(A12,'Margin Calculator'!$F$6:$F$8,1)),"Out of range")</f>
-        <v>Large</v>
+        <v>Full-Time</v>
       </c>
       <c r="C12" s="28" t="n">
         <f aca="false">IF(AND(A12&gt;='Margin Calculator'!$F$6,A12&lt;='Margin Calculator'!$G$8),INDEX('Margin Calculator'!$H$6:$H$8,MATCH(A12,'Margin Calculator'!$F$6:$F$8,1)),0)</f>
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D12" s="28" t="n">
         <f aca="false">A12*C12*'Margin Calculator'!$B$10/12</f>
-        <v>29293.3333333333</v>
+        <v>30160</v>
       </c>
       <c r="E12" s="28" t="n">
         <f aca="false">'Margin Calculator'!$B$6*A12*'Margin Calculator'!$B$9*'Margin Calculator'!$B$10/12</f>
@@ -1834,11 +1834,11 @@
       </c>
       <c r="G12" s="28" t="n">
         <f aca="false">D12-E12-F12</f>
-        <v>11093.3333333333</v>
+        <v>11960</v>
       </c>
       <c r="H12" s="29" t="n">
         <f aca="false">IFERROR(G12/D12,0)</f>
-        <v>0.378698224852071</v>
+        <v>0.396551724137931</v>
       </c>
       <c r="I12" s="28" t="n">
         <f aca="false">IFERROR(('Margin Calculator'!$B$6+'Margin Calculator'!$B$7)*'Margin Calculator'!$B$9/(1-'Margin Calculator'!$B$8),0)</f>

</xml_diff>